<commit_message>
Complete Exercise 4A inserts and update workbook
</commit_message>
<xml_diff>
--- a/Aweke_Ex3A_tables.xlsx
+++ b/Aweke_Ex3A_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/netsanetaweke/Documents/DATA_Labs/W2_Workshop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\netsaaweke\Documents\GitHub\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CED439-4129-064F-A7B5-89D8AA2C6537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03CF861-EF6C-4E0E-A790-07FD323A1F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4160" windowWidth="20640" windowHeight="17180" activeTab="4" xr2:uid="{3EA24EB7-6282-6D48-B925-3FCB11182F8D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{3EA24EB7-6282-6D48-B925-3FCB11182F8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
   <si>
     <t>Customer</t>
   </si>
@@ -118,13 +118,58 @@
   </si>
   <si>
     <t>Dog ID</t>
+  </si>
+  <si>
+    <t>Ephi Yoha</t>
+  </si>
+  <si>
+    <t>510-555-0101</t>
+  </si>
+  <si>
+    <t>Ephi@gmail.com</t>
+  </si>
+  <si>
+    <t>Buchu</t>
+  </si>
+  <si>
+    <t>Labrador</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Keep on leash</t>
+  </si>
+  <si>
+    <t>Sol Kidane</t>
+  </si>
+  <si>
+    <t>510-555-0102</t>
+  </si>
+  <si>
+    <t>Sol@gmail.com</t>
+  </si>
+  <si>
+    <t>1014 Street</t>
+  </si>
+  <si>
+    <t>Avenue</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Complete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -137,6 +182,14 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -168,16 +221,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -510,14 +569,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EB86823-F17F-E74D-9C20-70B66A40D48E}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.6328125" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="5" max="5" width="14.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -534,22 +595,42 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{FCF28936-BFDC-42E5-AD41-35FA620F4D05}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{616C26D0-94AE-CB45-A444-93F86E72DFEE}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="19.6328125" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -567,6 +648,26 @@
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -576,14 +677,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B500B9C6-1BD0-8A4D-8B08-4E56CE0782BE}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15.36328125" customWidth="1"/>
+    <col min="2" max="2" width="14.36328125" customWidth="1"/>
+    <col min="4" max="4" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -600,22 +702,42 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{3DDB8E4A-5947-4539-9CFA-FB86FE7FC6DC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8ADDD7D-E884-7E4F-AD92-4C1391FD8D4A}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
-    <col min="4" max="4" width="20.5" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -632,6 +754,26 @@
         <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46312</v>
+      </c>
+      <c r="C2">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
     </row>
@@ -642,14 +784,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F0E916-5CF1-AD4C-A6AE-4ED7E71546CD}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.6328125" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -670,6 +812,29 @@
       </c>
       <c r="G1" s="3" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6">
+        <v>46318</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.375</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>